<commit_message>
Ganti contoh data manual agar tidak menyalin referensi
</commit_message>
<xml_diff>
--- a/test-files/butircerdas-uji-10-soal-15-responden.xlsx
+++ b/test-files/butircerdas-uji-10-soal-15-responden.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriks" sheetId="1" r:id="R181256242a314ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriks" sheetId="1" r:id="Rde2afc94b06e4fff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -220,7 +220,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="5.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="5.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="2.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="2.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="2.380000114440918" hidden="0" customWidth="1"/>
@@ -270,7 +270,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>Ayu</x:v>
+        <x:v>Raka</x:v>
       </x:c>
       <x:c r="B2" s="4" t="n">
         <x:v>1</x:v>
@@ -279,25 +279,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D2" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F2" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H2" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I2" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J2" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K2" s="4" t="n">
         <x:v>1</x:v>
@@ -305,34 +305,34 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Bima</x:v>
+        <x:v>Salsa</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F3" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G3" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H3" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I3" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J3" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K3" s="4" t="n">
         <x:v>1</x:v>
@@ -340,10 +340,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="4" t="str">
-        <x:v>Cici</x:v>
+        <x:v>Naufal</x:v>
       </x:c>
       <x:c r="B4" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C4" s="4" t="n">
         <x:v>1</x:v>
@@ -352,7 +352,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="4" t="n">
         <x:v>1</x:v>
@@ -361,7 +361,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H4" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="4" t="n">
         <x:v>1</x:v>
@@ -370,39 +370,39 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K4" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="str">
-        <x:v>Dedi</x:v>
+        <x:v>Tania</x:v>
       </x:c>
       <x:c r="B5" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H5" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J5" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K5" s="4" t="n">
         <x:v>0</x:v>
@@ -410,10 +410,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="4" t="str">
-        <x:v>Eka</x:v>
+        <x:v>Bagas</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
         <x:v>0</x:v>
@@ -428,16 +428,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I6" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K6" s="4" t="n">
         <x:v>1</x:v>
@@ -445,10 +445,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="4" t="str">
-        <x:v>Fajar</x:v>
+        <x:v>Meisya</x:v>
       </x:c>
       <x:c r="B7" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
         <x:v>0</x:v>
@@ -457,19 +457,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F7" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H7" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I7" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="4" t="n">
         <x:v>0</x:v>
@@ -480,7 +480,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="4" t="str">
-        <x:v>Gina</x:v>
+        <x:v>Reno</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
         <x:v>1</x:v>
@@ -492,22 +492,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H8" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I8" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J8" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K8" s="4" t="n">
         <x:v>1</x:v>
@@ -515,25 +515,25 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="4" t="str">
-        <x:v>Hana</x:v>
+        <x:v>Dinda</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="4" t="n">
         <x:v>0</x:v>
@@ -542,7 +542,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K9" s="4" t="n">
         <x:v>1</x:v>
@@ -550,10 +550,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="4" t="str">
-        <x:v>Indra</x:v>
+        <x:v>Arman</x:v>
       </x:c>
       <x:c r="B10" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="4" t="n">
         <x:v>0</x:v>
@@ -562,16 +562,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H10" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I10" s="4" t="n">
         <x:v>0</x:v>
@@ -585,7 +585,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="4" t="str">
-        <x:v>Jihan</x:v>
+        <x:v>Putri</x:v>
       </x:c>
       <x:c r="B11" s="4" t="n">
         <x:v>1</x:v>
@@ -597,22 +597,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K11" s="4" t="n">
         <x:v>1</x:v>
@@ -620,7 +620,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="4" t="str">
-        <x:v>Kiki</x:v>
+        <x:v>Yusuf</x:v>
       </x:c>
       <x:c r="B12" s="4" t="n">
         <x:v>0</x:v>
@@ -635,13 +635,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I12" s="4" t="n">
         <x:v>1</x:v>
@@ -655,7 +655,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="4" t="str">
-        <x:v>Lala</x:v>
+        <x:v>Clara</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
         <x:v>1</x:v>
@@ -664,13 +664,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F13" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="4" t="n">
         <x:v>1</x:v>
@@ -679,10 +679,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I13" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J13" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K13" s="4" t="n">
         <x:v>1</x:v>
@@ -690,10 +690,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="4" t="str">
-        <x:v>Mira</x:v>
+        <x:v>Rizky</x:v>
       </x:c>
       <x:c r="B14" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="4" t="n">
         <x:v>0</x:v>
@@ -702,7 +702,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F14" s="4" t="n">
         <x:v>1</x:v>
@@ -714,7 +714,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I14" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J14" s="4" t="n">
         <x:v>0</x:v>
@@ -725,7 +725,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="4" t="str">
-        <x:v>Nina</x:v>
+        <x:v>Nabila</x:v>
       </x:c>
       <x:c r="B15" s="4" t="n">
         <x:v>1</x:v>
@@ -740,7 +740,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F15" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="4" t="n">
         <x:v>1</x:v>
@@ -755,12 +755,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K15" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="4" t="str">
-        <x:v>Oki</x:v>
+        <x:v>Farhan</x:v>
       </x:c>
       <x:c r="B16" s="4" t="n">
         <x:v>0</x:v>
@@ -769,7 +769,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="4" t="n">
         <x:v>0</x:v>
@@ -781,13 +781,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H16" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I16" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J16" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K16" s="4" t="n">
         <x:v>0</x:v>

</xml_diff>